<commit_message>
chore: added GUI annotation tools
</commit_message>
<xml_diff>
--- a/data/Truth.xlsx
+++ b/data/Truth.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Dropbox\AI Projects\otter\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9BF0F2F9-8BFF-48A6-9257-612E5E2A238A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13000B91-A48C-46B0-ACD9-DD3CDFD845A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="33435" yWindow="0" windowWidth="18525" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView minimized="1" xWindow="-45" yWindow="5565" windowWidth="19320" windowHeight="9690" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -8984,7 +8984,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="146" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:18" hidden="1" x14ac:dyDescent="0.25">
       <c r="A146" s="1" t="s">
         <v>163</v>
       </c>
@@ -9041,7 +9041,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="147" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:18" hidden="1" x14ac:dyDescent="0.25">
       <c r="A147" s="1" t="s">
         <v>162</v>
       </c>
@@ -9098,7 +9098,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="148" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:18" hidden="1" x14ac:dyDescent="0.25">
       <c r="A148" s="1" t="s">
         <v>164</v>
       </c>
@@ -9155,7 +9155,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="149" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:18" hidden="1" x14ac:dyDescent="0.25">
       <c r="A149" s="1" t="s">
         <v>165</v>
       </c>
@@ -9212,7 +9212,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="150" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:18" hidden="1" x14ac:dyDescent="0.25">
       <c r="A150" s="1" t="s">
         <v>166</v>
       </c>
@@ -9269,7 +9269,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="151" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:18" hidden="1" x14ac:dyDescent="0.25">
       <c r="A151" s="1" t="s">
         <v>167</v>
       </c>
@@ -9326,7 +9326,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="152" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:18" hidden="1" x14ac:dyDescent="0.25">
       <c r="A152" s="1" t="s">
         <v>168</v>
       </c>
@@ -9383,7 +9383,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="153" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:18" hidden="1" x14ac:dyDescent="0.25">
       <c r="A153" s="1" t="s">
         <v>169</v>
       </c>
@@ -9440,7 +9440,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="154" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:18" hidden="1" x14ac:dyDescent="0.25">
       <c r="A154" s="1" t="s">
         <v>170</v>
       </c>
@@ -9497,7 +9497,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="155" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:18" hidden="1" x14ac:dyDescent="0.25">
       <c r="A155" s="1" t="s">
         <v>171</v>
       </c>
@@ -9554,7 +9554,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="156" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:18" hidden="1" x14ac:dyDescent="0.25">
       <c r="A156" s="1" t="s">
         <v>172</v>
       </c>
@@ -9611,7 +9611,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="157" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:18" hidden="1" x14ac:dyDescent="0.25">
       <c r="A157" s="1" t="s">
         <v>173</v>
       </c>
@@ -9668,7 +9668,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="158" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:18" hidden="1" x14ac:dyDescent="0.25">
       <c r="A158" s="1" t="s">
         <v>174</v>
       </c>
@@ -9725,7 +9725,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="159" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:18" hidden="1" x14ac:dyDescent="0.25">
       <c r="A159" s="1" t="s">
         <v>175</v>
       </c>
@@ -10486,7 +10486,7 @@
         <v>0</v>
       </c>
       <c r="G172" s="1">
-        <f t="shared" ref="G172:G188" si="8">SUM(E172:F172)</f>
+        <f t="shared" ref="G172:G186" si="8">SUM(E172:F172)</f>
         <v>0</v>
       </c>
       <c r="H172" s="1">

</xml_diff>